<commit_message>
FEAT(hk212): okapní chodník complete 10-layer technology stack (#1240)
Okapní chodník po obvodu haly (0.7 m × 80 m, mimo 4 vstupy) — complete
10-item technology stack per ČSN 73 6126 + ČSN EN 13670 (řez A103 showed
only concrete profile — DPS gap).

Final stack (technological order):
  1. M-VK-027 Výkop rýhy 400 mm (22.4 m³)
  2. M-VK-028 Odvoz zeminy (22.4 m³)
  3. M-VK-024 Úprava + hutnění zemní pláně (56 m²)
  4. M-VK-029 Geotextilie 300 g/m² separační (56 m²)
  5. M-VK-022 Štěrk ŠD 32/63 150 mm (8.4 m³)
  6. M-VK-025 Hutnění štěrku (56 m²)
  7. M-VK-026 Bednění vnější hrana (16 m²)
  8. M-VK-021 KARI Q188 (56 m²)
  9. M-VK-020 Beton C25/30 XF3 200 mm (11.2 m³)
  10. M-VK-023 Dilatace á 4 m (20 m)

items.json 173 → 179. M-VK-021 de-bundled (KARI only). ABMV_32 open
(podkladní vrstvy verification — projektant Volka). 2 commits squashed.

https://claude.ai/code/session_016G4M9qpCUef7ZrVV6cJopc
</commit_message>
<xml_diff>
--- a/test-data/hk212_hala/outputs/sequential_list/hk212_sequential_list.xlsx
+++ b/test-data/hk212_hala/outputs/sequential_list/hk212_sequential_list.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J270"/>
+  <dimension ref="A1:J276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7329,7 +7329,7 @@
     <row r="254">
       <c r="A254" s="3" t="inlineStr">
         <is>
-          <t>→ Drcený štěrk podklady (rampy + okapní chodník)</t>
+          <t>→ Drcený štěrk podklad ramp</t>
         </is>
       </c>
     </row>
@@ -7372,356 +7372,441 @@
       <c r="J255" s="6" t="inlineStr"/>
     </row>
     <row r="256">
-      <c r="A256" s="10" t="n">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>→ Okapní chodník — complete 10-layer stack 0.7 m × 80 m po obvodu haly (výkop → odvoz → pláň → geotextilie → štěrk → hutnění → bednění → výztuž → beton → dilatace, pending ABMV_31 + ABMV_32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="4" t="n">
         <v>159</v>
       </c>
-      <c r="B256" s="11" t="inlineStr"/>
-      <c r="C256" s="10" t="n">
+      <c r="B257" s="5" t="inlineStr"/>
+      <c r="C257" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="D256" s="11" t="inlineStr">
+      <c r="D257" s="5" t="inlineStr">
         <is>
           <t>M-VK</t>
         </is>
       </c>
-      <c r="E256" s="11" t="inlineStr">
+      <c r="E257" s="5" t="inlineStr">
+        <is>
+          <t>M-VK-027</t>
+        </is>
+      </c>
+      <c r="F257" s="6" t="inlineStr">
+        <is>
+          <t>Výkop rýhy pro okapní chodník hl. 400 mm (na hloubku všech vrstev)</t>
+        </is>
+      </c>
+      <c r="G257" s="4" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="H257" s="4" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="I257" s="6" t="inlineStr">
+        <is>
+          <t>80.0 × 0.7 × 0.4 = 22.4 m³  [document:A103 řez A-B detail, norma:ČSN 73 6126, norma:ČSN okapový chodník]</t>
+        </is>
+      </c>
+      <c r="J257" s="6" t="inlineStr">
+        <is>
+          <t>ABMV:ABMV_32</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="10" t="n">
+        <v>160</v>
+      </c>
+      <c r="B258" s="11" t="inlineStr"/>
+      <c r="C258" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D258" s="11" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E258" s="11" t="inlineStr">
+        <is>
+          <t>M-VK-028</t>
+        </is>
+      </c>
+      <c r="F258" s="12" t="inlineStr">
+        <is>
+          <t>Odvoz vykopané zeminy z rýhy okapního chodníku na skládku</t>
+        </is>
+      </c>
+      <c r="G258" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="H258" s="10" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="I258" s="12">
+        <f> 22.4 m³ (1:1 s výkopem)  [document:A103 řez A-B detail, norma:ČSN 73 6126, norma:ČSN okapový chodník]</f>
+        <v/>
+      </c>
+      <c r="J258" s="12" t="inlineStr">
+        <is>
+          <t>ABMV:ABMV_32</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="4" t="n">
+        <v>161</v>
+      </c>
+      <c r="B259" s="5" t="inlineStr"/>
+      <c r="C259" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D259" s="5" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E259" s="5" t="inlineStr">
+        <is>
+          <t>M-VK-024</t>
+        </is>
+      </c>
+      <c r="F259" s="6" t="inlineStr">
+        <is>
+          <t>Úprava zemní pláně + hutnění pod okapní chodník (Edef2 ≥ 30 MPa)</t>
+        </is>
+      </c>
+      <c r="G259" s="4" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H259" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="I259" s="6" t="inlineStr">
+        <is>
+          <t>80.0 × 0.7 = 56.0 m²  [document:A103 řez A-B detail, norma:ČSN 73 6126, norma:ČSN EN 13670]</t>
+        </is>
+      </c>
+      <c r="J259" s="6" t="inlineStr">
+        <is>
+          <t>ABMV:ABMV_32</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="10" t="n">
+        <v>162</v>
+      </c>
+      <c r="B260" s="11" t="inlineStr"/>
+      <c r="C260" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D260" s="11" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E260" s="11" t="inlineStr">
+        <is>
+          <t>M-VK-029</t>
+        </is>
+      </c>
+      <c r="F260" s="12" t="inlineStr">
+        <is>
+          <t>Geotextilie 300 g/m² separační — mezi hutněnou zemní pláň a štěrkový podklad okapního chodníku</t>
+        </is>
+      </c>
+      <c r="G260" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H260" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="I260" s="12" t="inlineStr">
+        <is>
+          <t>80.0 × 0.7 = 56.0 m²  [document:A103 řez A-B detail, norma:ČSN 73 6126, norma:ČSN okapový chodník]</t>
+        </is>
+      </c>
+      <c r="J260" s="12" t="inlineStr">
+        <is>
+          <t>ABMV:ABMV_32</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="4" t="n">
+        <v>163</v>
+      </c>
+      <c r="B261" s="5" t="inlineStr"/>
+      <c r="C261" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D261" s="5" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E261" s="5" t="inlineStr">
         <is>
           <t>M-VK-022</t>
         </is>
       </c>
-      <c r="F256" s="12" t="inlineStr">
+      <c r="F261" s="6" t="inlineStr">
         <is>
           <t>Drcený štěrk ŠD 32/63 podklad okapního chodníku tl 150 mm</t>
         </is>
       </c>
-      <c r="G256" s="10" t="inlineStr">
+      <c r="G261" s="4" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="H256" s="10" t="n">
+      <c r="H261" s="4" t="n">
         <v>8.4</v>
       </c>
-      <c r="I256" s="12" t="inlineStr">
+      <c r="I261" s="6" t="inlineStr">
         <is>
           <t>80.0 × 0.7 × 0.15 = 8.40 m³  [document:A103 řezy A-B detail, document:A101 půdorys 1NP, document:C.3 KOO situace]</t>
         </is>
       </c>
-      <c r="J256" s="12" t="inlineStr">
+      <c r="J261" s="6" t="inlineStr">
         <is>
           <t>ABMV:ABMV_31</t>
         </is>
       </c>
     </row>
-    <row r="257">
-      <c r="A257" s="3" t="inlineStr">
-        <is>
-          <t>→ Okapní chodník — sokl 0.7 m × 80 m po obvodu haly (beton + výztuž + dilatace, pending ABMV_31)</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="B258" s="5" t="inlineStr"/>
-      <c r="C258" s="4" t="n">
+    <row r="262">
+      <c r="A262" s="10" t="n">
+        <v>164</v>
+      </c>
+      <c r="B262" s="11" t="inlineStr"/>
+      <c r="C262" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D258" s="5" t="inlineStr">
+      <c r="D262" s="11" t="inlineStr">
         <is>
           <t>M-VK</t>
         </is>
       </c>
-      <c r="E258" s="5" t="inlineStr">
+      <c r="E262" s="11" t="inlineStr">
+        <is>
+          <t>M-VK-025</t>
+        </is>
+      </c>
+      <c r="F262" s="12" t="inlineStr">
+        <is>
+          <t>Hutnění štěrkového podkladu okapního chodníku vibrodeskou (Edef2 ≥ 45 MPa)</t>
+        </is>
+      </c>
+      <c r="G262" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H262" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="I262" s="12" t="inlineStr">
+        <is>
+          <t>80.0 × 0.7 = 56.0 m²  [document:A103 řez A-B detail, norma:ČSN 73 6126, norma:ČSN EN 13670]</t>
+        </is>
+      </c>
+      <c r="J262" s="12" t="inlineStr">
+        <is>
+          <t>ABMV:ABMV_32</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="4" t="n">
+        <v>165</v>
+      </c>
+      <c r="B263" s="5" t="inlineStr"/>
+      <c r="C263" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D263" s="5" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E263" s="5" t="inlineStr">
+        <is>
+          <t>M-VK-026</t>
+        </is>
+      </c>
+      <c r="F263" s="6" t="inlineStr">
+        <is>
+          <t>Bednění boční vnější hrana okapního chodníku v 200 mm (vnitřní hrana = stěna haly)</t>
+        </is>
+      </c>
+      <c r="G263" s="4" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H263" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I263" s="6" t="inlineStr">
+        <is>
+          <t>80.0 × 0.2 = 16.0 m²  [document:A103 řez A-B detail, norma:ČSN 73 6126, norma:ČSN EN 13670]</t>
+        </is>
+      </c>
+      <c r="J263" s="6" t="inlineStr">
+        <is>
+          <t>ABMV:ABMV_32</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="10" t="n">
+        <v>166</v>
+      </c>
+      <c r="B264" s="11" t="inlineStr"/>
+      <c r="C264" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D264" s="11" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E264" s="11" t="inlineStr">
+        <is>
+          <t>M-VK-021</t>
+        </is>
+      </c>
+      <c r="F264" s="12" t="inlineStr">
+        <is>
+          <t>Výztuž KARI síť Q188 (150/150/6 mm) — okapní chodník</t>
+        </is>
+      </c>
+      <c r="G264" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H264" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="I264" s="12" t="inlineStr">
+        <is>
+          <t>80.0 × 0.7 = 56.00 m²  [document:A103 řezy A-B detail, document:A101 půdorys 1NP, document:C.3 KOO situace]</t>
+        </is>
+      </c>
+      <c r="J264" s="12" t="inlineStr">
+        <is>
+          <t>ABMV:ABMV_31</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="n">
+        <v>167</v>
+      </c>
+      <c r="B265" s="5" t="inlineStr"/>
+      <c r="C265" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D265" s="5" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E265" s="5" t="inlineStr">
         <is>
           <t>M-VK-020</t>
         </is>
       </c>
-      <c r="F258" s="6" t="inlineStr">
+      <c r="F265" s="6" t="inlineStr">
         <is>
           <t>Beton C25/30 XF3 — okapní chodník po obvodu haly (sokl 0.7 m × ~80 m mimo 4 vstupy), tl 200 mm</t>
         </is>
       </c>
-      <c r="G258" s="4" t="inlineStr">
+      <c r="G265" s="4" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="H258" s="4" t="n">
+      <c r="H265" s="4" t="n">
         <v>11.2</v>
       </c>
-      <c r="I258" s="6" t="inlineStr">
+      <c r="I265" s="6" t="inlineStr">
         <is>
           <t>80.0 × 0.7 × 0.2 = 11.20 m³  [document:A103 řezy A-B detail, document:A101 půdorys 1NP, document:C.3 KOO situace]</t>
         </is>
       </c>
-      <c r="J258" s="6" t="inlineStr">
+      <c r="J265" s="6" t="inlineStr">
         <is>
           <t>ABMV:ABMV_31</t>
         </is>
       </c>
     </row>
-    <row r="259">
-      <c r="A259" s="10" t="n">
-        <v>161</v>
-      </c>
-      <c r="B259" s="11" t="inlineStr"/>
-      <c r="C259" s="10" t="n">
+    <row r="266">
+      <c r="A266" s="10" t="n">
+        <v>168</v>
+      </c>
+      <c r="B266" s="11" t="inlineStr"/>
+      <c r="C266" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="D259" s="11" t="inlineStr">
+      <c r="D266" s="11" t="inlineStr">
         <is>
           <t>M-VK</t>
         </is>
       </c>
-      <c r="E259" s="11" t="inlineStr">
-        <is>
-          <t>M-VK-021</t>
-        </is>
-      </c>
-      <c r="F259" s="12" t="inlineStr">
-        <is>
-          <t>Výztuž KARI síť Q188 + boční bednění + dilatační lišty — okapní chodník</t>
-        </is>
-      </c>
-      <c r="G259" s="10" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="H259" s="10" t="n">
-        <v>56</v>
-      </c>
-      <c r="I259" s="12" t="inlineStr">
-        <is>
-          <t>80.0 × 0.7 = 56.00 m²  [document:A103 řezy A-B detail, document:A101 půdorys 1NP, document:C.3 KOO situace]</t>
-        </is>
-      </c>
-      <c r="J259" s="12" t="inlineStr">
+      <c r="E266" s="11" t="inlineStr">
+        <is>
+          <t>M-VK-023</t>
+        </is>
+      </c>
+      <c r="F266" s="12" t="inlineStr">
+        <is>
+          <t>Dilatační lišty + těsnění spár mezi segmenty okapního chodníku (à ~4 m)</t>
+        </is>
+      </c>
+      <c r="G266" s="10" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="H266" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="I266" s="12" t="inlineStr">
+        <is>
+          <t>80.0 / 4 = 20 ks dilatací  [document:A103 řezy A-B detail, document:A101 půdorys 1NP, document:C.3 KOO situace]</t>
+        </is>
+      </c>
+      <c r="J266" s="12" t="inlineStr">
         <is>
           <t>ABMV:ABMV_31</t>
         </is>
       </c>
-    </row>
-    <row r="260">
-      <c r="A260" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="B260" s="5" t="inlineStr"/>
-      <c r="C260" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D260" s="5" t="inlineStr">
-        <is>
-          <t>M-VK</t>
-        </is>
-      </c>
-      <c r="E260" s="5" t="inlineStr">
-        <is>
-          <t>M-VK-023</t>
-        </is>
-      </c>
-      <c r="F260" s="6" t="inlineStr">
-        <is>
-          <t>Dilatační lišty + těsnění spár mezi segmenty okapního chodníku (à ~4 m)</t>
-        </is>
-      </c>
-      <c r="G260" s="4" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="H260" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="I260" s="6" t="inlineStr">
-        <is>
-          <t>80.0 / 4 = 20 ks dilatací  [document:A103 řezy A-B detail, document:A101 půdorys 1NP, document:C.3 KOO situace]</t>
-        </is>
-      </c>
-      <c r="J260" s="6" t="inlineStr">
-        <is>
-          <t>ABMV:ABMV_31</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="3" t="inlineStr">
-        <is>
-          <t>→ Rampy 4× (R1-R4) — výztuž + bednění + beton + obrubník (per A101)</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" s="4" t="n">
-        <v>163</v>
-      </c>
-      <c r="B262" s="5" t="inlineStr"/>
-      <c r="C262" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D262" s="5" t="inlineStr">
-        <is>
-          <t>M-VK</t>
-        </is>
-      </c>
-      <c r="E262" s="5" t="inlineStr">
-        <is>
-          <t>M-VK-002</t>
-        </is>
-      </c>
-      <c r="F262" s="6" t="inlineStr">
-        <is>
-          <t>Výztuž KARI síť Q188 + bednění boční rampy 4 lokality</t>
-        </is>
-      </c>
-      <c r="G262" s="4" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="H262" s="4" t="n">
-        <v>43.32</v>
-      </c>
-      <c r="I262" s="6" t="inlineStr">
-        <is>
-          <t>4 lokality rampy = 43.32 m²  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
-        </is>
-      </c>
-      <c r="J262" s="6" t="inlineStr"/>
-    </row>
-    <row r="263">
-      <c r="A263" s="10" t="n">
-        <v>164</v>
-      </c>
-      <c r="B263" s="11" t="inlineStr"/>
-      <c r="C263" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D263" s="11" t="inlineStr">
-        <is>
-          <t>M-VK</t>
-        </is>
-      </c>
-      <c r="E263" s="11" t="inlineStr">
-        <is>
-          <t>M-VK-001</t>
-        </is>
-      </c>
-      <c r="F263" s="12" t="inlineStr">
-        <is>
-          <t>Beton C25/30 XF3 — vstupní/nájezdové rampy tl 150 mm, 4 lokality (R1 sever, R2+R3 jih, R4 západ bezbariérová)</t>
-        </is>
-      </c>
-      <c r="G263" s="10" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="H263" s="10" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="I263" s="12" t="inlineStr">
-        <is>
-          <t>(9.2+11.5+9.2+13.42) × 0.15 = 6.50 m³  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
-        </is>
-      </c>
-      <c r="J263" s="12" t="inlineStr"/>
-    </row>
-    <row r="264">
-      <c r="A264" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="B264" s="5" t="inlineStr"/>
-      <c r="C264" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D264" s="5" t="inlineStr">
-        <is>
-          <t>M-VK</t>
-        </is>
-      </c>
-      <c r="E264" s="5" t="inlineStr">
-        <is>
-          <t>M-VK-004</t>
-        </is>
-      </c>
-      <c r="F264" s="6" t="inlineStr">
-        <is>
-          <t>Obrubník betonový ABO 100×250×1000 kolem ramp + lůžko z betonu C16/20</t>
-        </is>
-      </c>
-      <c r="G264" s="4" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="H264" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="I264" s="6" t="inlineStr">
-        <is>
-          <t>~30.0 m  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
-        </is>
-      </c>
-      <c r="J264" s="6" t="inlineStr"/>
-    </row>
-    <row r="265">
-      <c r="A265" s="3" t="inlineStr">
-        <is>
-          <t>→ Liniový žlab pojízdný B125 — SZ + JZ fasáda (40 m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" s="4" t="n">
-        <v>166</v>
-      </c>
-      <c r="B266" s="5" t="inlineStr"/>
-      <c r="C266" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D266" s="5" t="inlineStr">
-        <is>
-          <t>M-VK</t>
-        </is>
-      </c>
-      <c r="E266" s="5" t="inlineStr">
-        <is>
-          <t>M-VK-012</t>
-        </is>
-      </c>
-      <c r="F266" s="6" t="inlineStr">
-        <is>
-          <t>Liniový žlab POJÍZDNÝ tř. zatížení B125 — odvodnění zpevněných ploch parkoviště + manipulace, vč. mřížky</t>
-        </is>
-      </c>
-      <c r="G266" s="4" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="H266" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="I266" s="6" t="inlineStr">
-        <is>
-          <t>40 m  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
-        </is>
-      </c>
-      <c r="J266" s="6" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
         <is>
-          <t>→ Vyspádování okolního terénu k odvodnění</t>
+          <t>→ Rampy 4× (R1-R4) — výztuž + bednění + beton + obrubník (per A101)</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B268" s="5" t="inlineStr"/>
       <c r="C268" s="4" t="n">
@@ -7734,12 +7819,12 @@
       </c>
       <c r="E268" s="5" t="inlineStr">
         <is>
-          <t>M-VK-019</t>
+          <t>M-VK-002</t>
         </is>
       </c>
       <c r="F268" s="6" t="inlineStr">
         <is>
-          <t>Vyspádování okolního terénu k odvodňovacím prvkům (žlabům, retenční nádrži) — hutněná zemina, finální úprava</t>
+          <t>Výztuž KARI síť Q188 + bednění boční rampy 4 lokality</t>
         </is>
       </c>
       <c r="G268" s="4" t="inlineStr">
@@ -7748,25 +7833,56 @@
         </is>
       </c>
       <c r="H268" s="4" t="n">
-        <v>300</v>
+        <v>43.32</v>
       </c>
       <c r="I268" s="6" t="inlineStr">
         <is>
-          <t>300 m²  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
+          <t>4 lokality rampy = 43.32 m²  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
         </is>
       </c>
       <c r="J268" s="6" t="inlineStr"/>
     </row>
     <row r="269">
-      <c r="A269" s="3" t="inlineStr">
-        <is>
-          <t>→ Ohumusování + osetí travou zbytkových ploch</t>
-        </is>
-      </c>
+      <c r="A269" s="10" t="n">
+        <v>170</v>
+      </c>
+      <c r="B269" s="11" t="inlineStr"/>
+      <c r="C269" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D269" s="11" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E269" s="11" t="inlineStr">
+        <is>
+          <t>M-VK-001</t>
+        </is>
+      </c>
+      <c r="F269" s="12" t="inlineStr">
+        <is>
+          <t>Beton C25/30 XF3 — vstupní/nájezdové rampy tl 150 mm, 4 lokality (R1 sever, R2+R3 jih, R4 západ bezbariérová)</t>
+        </is>
+      </c>
+      <c r="G269" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="H269" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I269" s="12" t="inlineStr">
+        <is>
+          <t>(9.2+11.5+9.2+13.42) × 0.15 = 6.50 m³  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
+        </is>
+      </c>
+      <c r="J269" s="12" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B270" s="5" t="inlineStr"/>
       <c r="C270" s="4" t="n">
@@ -7779,28 +7895,163 @@
       </c>
       <c r="E270" s="5" t="inlineStr">
         <is>
+          <t>M-VK-004</t>
+        </is>
+      </c>
+      <c r="F270" s="6" t="inlineStr">
+        <is>
+          <t>Obrubník betonový ABO 100×250×1000 kolem ramp + lůžko z betonu C16/20</t>
+        </is>
+      </c>
+      <c r="G270" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="H270" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I270" s="6" t="inlineStr">
+        <is>
+          <t>~30.0 m  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
+        </is>
+      </c>
+      <c r="J270" s="6" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="3" t="inlineStr">
+        <is>
+          <t>→ Liniový žlab pojízdný B125 — SZ + JZ fasáda (40 m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="4" t="n">
+        <v>172</v>
+      </c>
+      <c r="B272" s="5" t="inlineStr"/>
+      <c r="C272" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D272" s="5" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E272" s="5" t="inlineStr">
+        <is>
+          <t>M-VK-012</t>
+        </is>
+      </c>
+      <c r="F272" s="6" t="inlineStr">
+        <is>
+          <t>Liniový žlab POJÍZDNÝ tř. zatížení B125 — odvodnění zpevněných ploch parkoviště + manipulace, vč. mřížky</t>
+        </is>
+      </c>
+      <c r="G272" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="H272" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="I272" s="6" t="inlineStr">
+        <is>
+          <t>40 m  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
+        </is>
+      </c>
+      <c r="J272" s="6" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="3" t="inlineStr">
+        <is>
+          <t>→ Vyspádování okolního terénu k odvodnění</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="B274" s="5" t="inlineStr"/>
+      <c r="C274" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D274" s="5" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E274" s="5" t="inlineStr">
+        <is>
+          <t>M-VK-019</t>
+        </is>
+      </c>
+      <c r="F274" s="6" t="inlineStr">
+        <is>
+          <t>Vyspádování okolního terénu k odvodňovacím prvkům (žlabům, retenční nádrži) — hutněná zemina, finální úprava</t>
+        </is>
+      </c>
+      <c r="G274" s="4" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H274" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I274" s="6" t="inlineStr">
+        <is>
+          <t>300 m²  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
+        </is>
+      </c>
+      <c r="J274" s="6" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="3" t="inlineStr">
+        <is>
+          <t>→ Ohumusování + osetí travou zbytkových ploch</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="4" t="n">
+        <v>174</v>
+      </c>
+      <c r="B276" s="5" t="inlineStr"/>
+      <c r="C276" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D276" s="5" t="inlineStr">
+        <is>
+          <t>M-VK</t>
+        </is>
+      </c>
+      <c r="E276" s="5" t="inlineStr">
+        <is>
           <t>M-VK-018</t>
         </is>
       </c>
-      <c r="F270" s="6" t="inlineStr">
+      <c r="F276" s="6" t="inlineStr">
         <is>
           <t>Ohumusování tl 100 mm + osetí trávou parkové směsi — rekultivace zbytkových ploch okolo haly</t>
         </is>
       </c>
-      <c r="G270" s="4" t="inlineStr">
+      <c r="G276" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H270" s="4" t="n">
+      <c r="H276" s="4" t="n">
         <v>500</v>
       </c>
-      <c r="I270" s="6" t="inlineStr">
+      <c r="I276" s="6" t="inlineStr">
         <is>
           <t>500 m²  [document:C.3 KOO situace, document:A101 půdorys 1NP, document:A103 řez A-B]</t>
         </is>
       </c>
-      <c r="J270" s="6" t="inlineStr"/>
+      <c r="J276" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="101">
@@ -7813,7 +8064,6 @@
     <mergeCell ref="A220:J220"/>
     <mergeCell ref="A34:J34"/>
     <mergeCell ref="A83:J83"/>
-    <mergeCell ref="A261:J261"/>
     <mergeCell ref="A222:J222"/>
     <mergeCell ref="A49:J49"/>
     <mergeCell ref="A138:J138"/>
@@ -7821,6 +8071,7 @@
     <mergeCell ref="A36:J36"/>
     <mergeCell ref="A6:J6"/>
     <mergeCell ref="A119:J119"/>
+    <mergeCell ref="A256:J256"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A95:J95"/>
     <mergeCell ref="A248:J248"/>
@@ -7828,15 +8079,14 @@
     <mergeCell ref="A159:J159"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A96:J96"/>
-    <mergeCell ref="A265:J265"/>
     <mergeCell ref="A147:J147"/>
     <mergeCell ref="A121:J121"/>
     <mergeCell ref="A202:J202"/>
     <mergeCell ref="A58:J58"/>
     <mergeCell ref="A186:J186"/>
-    <mergeCell ref="A257:J257"/>
     <mergeCell ref="A24:J24"/>
     <mergeCell ref="A201:J201"/>
+    <mergeCell ref="A275:J275"/>
     <mergeCell ref="A250:J250"/>
     <mergeCell ref="A197:J197"/>
     <mergeCell ref="A110:J110"/>
@@ -7880,7 +8130,6 @@
     <mergeCell ref="A33:J33"/>
     <mergeCell ref="A85:J85"/>
     <mergeCell ref="A116:J116"/>
-    <mergeCell ref="A269:J269"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="A188:J188"/>
     <mergeCell ref="A126:J126"/>
@@ -7895,11 +8144,13 @@
     <mergeCell ref="A232:J232"/>
     <mergeCell ref="A142:J142"/>
     <mergeCell ref="A216:J216"/>
+    <mergeCell ref="A271:J271"/>
     <mergeCell ref="A65:J65"/>
     <mergeCell ref="A218:J218"/>
     <mergeCell ref="A193:J193"/>
     <mergeCell ref="A80:J80"/>
     <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A273:J273"/>
     <mergeCell ref="A89:J89"/>
     <mergeCell ref="A57:J57"/>
     <mergeCell ref="A235:J235"/>

</xml_diff>